<commit_message>
Deployment fix: Enable environment-based API URL and Render support
</commit_message>
<xml_diff>
--- a/backend/attendance.xlsx
+++ b/backend/attendance.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L17"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -924,9 +924,85 @@
         <v>24</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B16" t="str">
+        <v>6:19:05 pm</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Nagar</v>
+      </c>
+      <c r="D16" t="str">
+        <v>hr54ab3456</v>
+      </c>
+      <c r="E16" t="str">
+        <v>testing</v>
+      </c>
+      <c r="F16" t="str">
+        <v>4563256987</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="H16" t="str">
+        <v>No</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Bolero</v>
+      </c>
+      <c r="J16">
+        <v>28.375835240533487</v>
+      </c>
+      <c r="K16">
+        <v>77.07727009614061</v>
+      </c>
+      <c r="L16">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-04-14</v>
+      </c>
+      <c r="B17" t="str">
+        <v>6:24:04 pm</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Blue Wheel</v>
+      </c>
+      <c r="D17" t="str">
+        <v>MH56AB5678</v>
+      </c>
+      <c r="E17" t="str">
+        <v>testing2</v>
+      </c>
+      <c r="F17" t="str">
+        <v>7854698523</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Eeco</v>
+      </c>
+      <c r="J17">
+        <v>28.375945410830017</v>
+      </c>
+      <c r="K17">
+        <v>77.07712784118003</v>
+      </c>
+      <c r="L17">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>